<commit_message>
paper run 2026-09-09 17:55
</commit_message>
<xml_diff>
--- a/reports/2026-09-09.xlsx
+++ b/reports/2026-09-09.xlsx
@@ -571,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -743,13 +743,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D16" t="n">
-        <v>22.61</v>
+        <v>167.72</v>
       </c>
       <c r="E16" t="n">
         <v>10.92</v>
@@ -803,7 +803,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -813,7 +813,7 @@
         <v>1</v>
       </c>
       <c r="D20" t="n">
-        <v>18.82</v>
+        <v>40.07</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -822,421 +822,440 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>4</v>
+      </c>
+      <c r="C21" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" t="n">
+        <v>123.86</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>1</v>
-      </c>
-      <c r="C22" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" t="n">
-        <v>-39.88</v>
-      </c>
-      <c r="E22" t="n">
-        <v>-7.2</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D23" t="n">
-        <v>41.43</v>
+        <v>105.23</v>
       </c>
       <c r="E23" t="n">
-        <v>10.92</v>
+        <v>-7.2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" t="n">
+        <v>41.43</v>
+      </c>
+      <c r="E24" t="n">
+        <v>10.92</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>1</v>
-      </c>
-      <c r="C25" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" t="n">
-        <v>18.82</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0</v>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>5</v>
+      </c>
+      <c r="C26" t="n">
+        <v>5</v>
+      </c>
+      <c r="D26" t="n">
+        <v>163.93</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B26" t="n">
+      <c r="B27" t="n">
         <v>2</v>
       </c>
-      <c r="C26" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" t="n">
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" t="n">
         <v>-17.27</v>
       </c>
-      <c r="E26" t="n">
+      <c r="E27" t="n">
         <v>3.72</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>REALIZED (реальные сделки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>BTC</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>1</v>
-      </c>
-      <c r="C31" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" t="n">
-        <v>-7.2</v>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" t="n">
+        <v>-7.2</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>ETH</t>
         </is>
       </c>
-      <c r="B32" t="n">
-        <v>1</v>
-      </c>
-      <c r="C32" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" t="n">
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
         <v>10.92</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>15m</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" t="n">
-        <v>0</v>
-      </c>
-      <c r="D35" t="n">
-        <v>-7.2</v>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" t="n">
+        <v>-7.2</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>5m</t>
         </is>
       </c>
-      <c r="B36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C36" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" t="n">
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
         <v>10.92</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>1</v>
-      </c>
-      <c r="C39" t="n">
-        <v>0</v>
-      </c>
-      <c r="D39" t="n">
-        <v>-7.2</v>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" t="n">
+        <v>-7.2</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>04</t>
         </is>
       </c>
-      <c r="B40" t="n">
-        <v>1</v>
-      </c>
-      <c r="C40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" t="n">
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
         <v>10.92</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>1</v>
-      </c>
-      <c r="C43" t="n">
-        <v>0</v>
-      </c>
-      <c r="D43" t="n">
-        <v>-7.2</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" t="n">
+        <v>-7.2</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>0.60–0.62</t>
         </is>
       </c>
-      <c r="B44" t="n">
-        <v>1</v>
-      </c>
-      <c r="C44" t="n">
-        <v>1</v>
-      </c>
-      <c r="D44" t="n">
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
         <v>10.92</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>1</v>
-      </c>
-      <c r="C47" t="n">
-        <v>0</v>
-      </c>
-      <c r="D47" t="n">
-        <v>-7.2</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" t="n">
+        <v>-7.2</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
           <t>0.15–0.20%</t>
         </is>
       </c>
-      <c r="B48" t="n">
-        <v>1</v>
-      </c>
-      <c r="C48" t="n">
-        <v>1</v>
-      </c>
-      <c r="D48" t="n">
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" t="n">
         <v>10.92</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>1</v>
-      </c>
-      <c r="C51" t="n">
-        <v>1</v>
-      </c>
-      <c r="D51" t="n">
-        <v>10.92</v>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" t="n">
+        <v>10.92</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B52" t="n">
-        <v>1</v>
-      </c>
-      <c r="C52" t="n">
+      <c r="B53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C53" t="n">
         <v>0</v>
       </c>
-      <c r="D52" t="n">
+      <c r="D53" t="n">
         <v>-7.2</v>
       </c>
     </row>

</xml_diff>